<commit_message>
Add BOQ PR Sheet to BOQ
</commit_message>
<xml_diff>
--- a/data/template/boq/BOQ Documentation.xlsx
+++ b/data/template/boq/BOQ Documentation.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JACOBS\SERVICE\API\data\template\boq\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8A2A263-974A-404F-B2E5-6E06898FFC61}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B00A3D2-B59D-4F51-B9A0-525EAD92B4B1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Save" sheetId="3" r:id="rId1"/>
-    <sheet name="Question" sheetId="5" r:id="rId2"/>
+    <sheet name="BOQ Sheet" sheetId="3" r:id="rId1"/>
+    <sheet name="BOQ PR Sheet" sheetId="6" r:id="rId2"/>
+    <sheet name="Question" sheetId="5" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1323" uniqueCount="859">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1389" uniqueCount="887">
   <si>
     <t>program</t>
   </si>
@@ -2598,6 +2599,93 @@
   </si>
   <si>
     <t>Test OTDR</t>
+  </si>
+  <si>
+    <t>Variable</t>
+  </si>
+  <si>
+    <t>num</t>
+  </si>
+  <si>
+    <t>permit</t>
+  </si>
+  <si>
+    <t>shop_incl_pole_aerial</t>
+  </si>
+  <si>
+    <t>shop_excl_pole_aerial</t>
+  </si>
+  <si>
+    <t>shop_burial</t>
+  </si>
+  <si>
+    <t>comcase</t>
+  </si>
+  <si>
+    <t>mat_pole_7</t>
+  </si>
+  <si>
+    <t>mat_pole_9</t>
+  </si>
+  <si>
+    <t>mat_cable_fo_24</t>
+  </si>
+  <si>
+    <t>mat_cable_fo_96</t>
+  </si>
+  <si>
+    <t>mat_hdpe</t>
+  </si>
+  <si>
+    <t>total_e2e_dist</t>
+  </si>
+  <si>
+    <t>pole_exist</t>
+  </si>
+  <si>
+    <t>Shopping List Pekerjaan FO Intersite 
+(Incl. Instalasi Pole) - Aerial (All In)</t>
+  </si>
+  <si>
+    <t>Shopping List Pekerjaan FO Intersite 
+(Excl. Instalasi Pole) - Aerial (All In)</t>
+  </si>
+  <si>
+    <t>Shopping List Pekerjaan FO Intersite
+- Burial (All In)</t>
+  </si>
+  <si>
+    <t>Comcase</t>
+  </si>
+  <si>
+    <t>Material HDPE</t>
+  </si>
+  <si>
+    <t>Pole Exist</t>
+  </si>
+  <si>
+    <t>Column</t>
+  </si>
+  <si>
+    <t>Material Pole 7</t>
+  </si>
+  <si>
+    <t>Material Pole 9</t>
+  </si>
+  <si>
+    <t>Material Kabel FO 24 C</t>
+  </si>
+  <si>
+    <t>Material Kabel FO 96 C</t>
+  </si>
+  <si>
+    <t>meter</t>
+  </si>
+  <si>
+    <t>Permit (Arial - Burial) All In</t>
+  </si>
+  <si>
+    <t>Formula berbeda di XL sama dengan material HDPE di Surge material/2</t>
   </si>
 </sst>
 </file>
@@ -2740,7 +2828,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2803,6 +2891,11 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -10233,6 +10326,264 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5863C4C0-30E9-48D3-B4AA-B4587F53915C}">
+  <dimension ref="A1:C22"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="71.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="27" t="s">
+        <v>879</v>
+      </c>
+      <c r="B1" s="27" t="s">
+        <v>464</v>
+      </c>
+      <c r="C1" s="27" t="s">
+        <v>859</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>432</v>
+      </c>
+      <c r="C2" s="29" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="28" t="s">
+        <v>432</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="28" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="28" t="s">
+        <v>432</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="28" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="28" t="s">
+        <v>432</v>
+      </c>
+      <c r="C5" s="29" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="28" t="s">
+        <v>432</v>
+      </c>
+      <c r="C6" s="29" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="28" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="28" t="s">
+        <v>432</v>
+      </c>
+      <c r="C7" s="29" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="28" t="s">
+        <v>432</v>
+      </c>
+      <c r="C8" s="29" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="28" t="s">
+        <v>432</v>
+      </c>
+      <c r="C9" s="29" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="28" t="s">
+        <v>432</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="28" t="s">
+        <v>885</v>
+      </c>
+      <c r="B11" s="28" t="s">
+        <v>884</v>
+      </c>
+      <c r="C11" s="29" t="s">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="28" t="s">
+        <v>873</v>
+      </c>
+      <c r="B12" s="28" t="s">
+        <v>884</v>
+      </c>
+      <c r="C12" s="29" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="28" t="s">
+        <v>874</v>
+      </c>
+      <c r="B13" s="28" t="s">
+        <v>884</v>
+      </c>
+      <c r="C13" s="29" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="28" t="s">
+        <v>875</v>
+      </c>
+      <c r="B14" s="28" t="s">
+        <v>884</v>
+      </c>
+      <c r="C14" s="29" t="s">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="28" t="s">
+        <v>876</v>
+      </c>
+      <c r="B15" s="28" t="s">
+        <v>884</v>
+      </c>
+      <c r="C15" s="29" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="28" t="s">
+        <v>880</v>
+      </c>
+      <c r="B16" s="28" t="s">
+        <v>463</v>
+      </c>
+      <c r="C16" s="29" t="s">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="28" t="s">
+        <v>881</v>
+      </c>
+      <c r="B17" s="28" t="s">
+        <v>463</v>
+      </c>
+      <c r="C17" s="29" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="28" t="s">
+        <v>882</v>
+      </c>
+      <c r="B18" s="28" t="s">
+        <v>884</v>
+      </c>
+      <c r="C18" s="29" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="28" t="s">
+        <v>883</v>
+      </c>
+      <c r="B19" s="28" t="s">
+        <v>884</v>
+      </c>
+      <c r="C19" s="29" t="s">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="28" t="s">
+        <v>877</v>
+      </c>
+      <c r="B20" s="28" t="s">
+        <v>884</v>
+      </c>
+      <c r="C20" s="29" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="28" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" s="28" t="s">
+        <v>884</v>
+      </c>
+      <c r="C21" s="29" t="s">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="28" t="s">
+        <v>878</v>
+      </c>
+      <c r="B22" s="28" t="s">
+        <v>884</v>
+      </c>
+      <c r="C22" s="29" t="s">
+        <v>872</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CA441E6-6BE3-4CCB-8299-2EEB305EB638}">
   <dimension ref="A2:B5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -10261,7 +10612,7 @@
         <v>857</v>
       </c>
       <c r="B4" t="s">
-        <v>854</v>
+        <v>886</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>